<commit_message>
demo: update fts forms.
</commit_message>
<xml_diff>
--- a/Demo/lf/demo_lf_tas_9999_3_fts.xlsx
+++ b/Demo/lf/demo_lf_tas_9999_3_fts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\lf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE38CC72-2E41-451E-9510-91F962FE500B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DAC5377-9B70-45A6-A2B9-4B96B35DC6C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="189">
   <si>
     <t>type</t>
   </si>
@@ -1887,7 +1887,9 @@
       <c r="C29" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="H29" s="38"/>
+      <c r="H29" s="29" t="s">
+        <v>106</v>
+      </c>
       <c r="I29" s="27"/>
     </row>
     <row r="30" spans="1:13">

</xml_diff>